<commit_message>
EPBDS-16842 Fix test tables rounding a BigDecimal result to a Double, which passed an expected value wrong after the 16th digit
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/4-Testing/TestTables.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/4-Testing/TestTables.xlsx
@@ -1650,13 +1650,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I96"/>
+  <dimension ref="B2:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="20.9" customWidth="1" min="3" max="3"/>
-    <col width="12.5" customWidth="1" min="4" max="4"/>
+    <col width="39.8" customWidth="1" min="4" max="4"/>
     <col width="14.6" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1825,7 +1825,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Precision: "_res_ (2)" compares a number with 2 decimal places, so the difference must be less than 0.01. The "precision" property sets it for the whole test table. A negative precision rounds to tens, hundreds and so on.</t>
+          <t>Precision: "_res_ (2)" compares a number with 2 decimal places, so the difference may be up to 0.01. The "precision" property sets it for the whole test table. A negative precision rounds to tens, hundreds and so on.</t>
         </is>
       </c>
     </row>
@@ -2263,165 +2263,307 @@
       </c>
       <c r="D72" s="6" t="n"/>
     </row>
-    <row r="74" ht="16.5" customHeight="1">
+    <row r="74" ht="30" customHeight="1">
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>A rule that returns Object is checked by the text of the value: "10" matches the number 10.0, the Integer 10 and the text "10".</t>
+          <t>A BigDecimal result is compared with all its digits. Two thirds is 0.6666666666666666666666666666666667 with 34 digits, and a shorter expected value does not match it. A precision allows a difference up to 1E-n, computed exactly: 0.6666666667 matches with "_res_ (10)".</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Method Object AnyValue(String kind)</t>
+          <t>Method BigDecimal Share(BigDecimal part, BigDecimal whole)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
         <is>
+          <t>return part / whole;</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Test Share ShareTest</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="n"/>
+      <c r="D79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>part</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>whole</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Whole</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>0.6666666666666666666666666666666667</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D83" s="7" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Test Share SharePrecisionTest</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="n"/>
+      <c r="D85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>part</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>whole</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>_res_ (10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Whole</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>0.6666666667</v>
+      </c>
+    </row>
+    <row r="90" ht="16.5" customHeight="1">
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>A rule that returns Object is checked by the text of the value: "10" matches the number 10.0, the Integer 10 and the text "10".</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Method Object AnyValue(String kind)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="6" t="inlineStr">
+        <is>
           <t>if (kind == "double") { return 10.0; }</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="B78" s="6" t="inlineStr">
+    <row r="94">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>if (kind == "integer") { return 10; }</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="B79" s="6" t="inlineStr">
+    <row r="95">
+      <c r="B95" s="6" t="inlineStr">
         <is>
           <t>if (kind == "array") { return new double[] {10.0}; }</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="B80" s="6" t="inlineStr">
+    <row r="96">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>return "10";</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="B82" s="3" t="inlineStr">
+    <row r="98">
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>Test AnyValue AnyValueTest</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n"/>
-    </row>
-    <row r="83">
-      <c r="B83" s="9" t="inlineStr">
+      <c r="C98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="9" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C83" s="9" t="inlineStr">
+      <c r="C99" s="9" t="inlineStr">
         <is>
           <t>_res_</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="B84" s="5" t="inlineStr">
+    <row r="100">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="6" t="inlineStr">
+    <row r="101">
+      <c r="B101" s="6" t="inlineStr">
         <is>
           <t>double</t>
         </is>
       </c>
-      <c r="C85" s="7" t="n">
+      <c r="C101" s="7" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="86">
-      <c r="B86" s="6" t="inlineStr">
+    <row r="102">
+      <c r="B102" s="6" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="C86" s="7" t="n">
+      <c r="C102" s="7" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="87">
-      <c r="B87" s="6" t="inlineStr">
+    <row r="103">
+      <c r="B103" s="6" t="inlineStr">
         <is>
           <t>array</t>
         </is>
       </c>
-      <c r="C87" s="7" t="n">
+      <c r="C103" s="7" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="88">
-      <c r="B88" s="6" t="inlineStr">
+    <row r="104">
+      <c r="B104" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="C88" s="7" t="n">
+      <c r="C104" s="7" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="90">
-      <c r="B90" s="3" t="inlineStr">
+    <row r="106">
+      <c r="B106" s="3" t="inlineStr">
         <is>
           <t>Method Object[] AnyArray()</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="B91" s="6" t="inlineStr">
+    <row r="107">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>return new int[] {10, 20};</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="B93" s="3" t="inlineStr">
+    <row r="109">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>Test AnyArray AnyArrayTest</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="B94" s="9" t="inlineStr">
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
         <is>
           <t>_res_</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="B95" s="5" t="inlineStr">
+    <row r="111">
+      <c r="B111" s="5" t="inlineStr">
         <is>
           <t>Values</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="B96" s="7" t="inlineStr">
+    <row r="112">
+      <c r="B112" s="7" t="inlineStr">
         <is>
           <t>10, 20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="B74:I74"/>
+  <mergeCells count="17">
+    <mergeCell ref="B90:I90"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B67:D67"/>
@@ -2431,10 +2573,13 @@
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B61:C61"/>
     <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B98:C98"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="B85:D85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>